<commit_message>
Chiller seti CH-1..5 IC SET'ten (calisanlarin ortak degeri); yanlis adresli CH SET (0103/AV12 = kollektor denetleyicisi) sablondan ve kopruden kaldirildi
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DrVFiyvjUKiEmUZQRoKZ5y
</commit_message>
<xml_diff>
--- a/hvac/deneme/configs/hedefli_okuma_sablonu_2.xlsx
+++ b/hvac/deneme/configs/hedefli_okuma_sablonu_2.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" windowWidth="27945" windowHeight="11325" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet1'!$A$1:$G$40</definedName>
@@ -1100,7 +1100,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G53"/>
+  <dimension ref="A1:G52"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
     <col width="13.2857142857143" customWidth="1" style="1" min="1" max="1"/>
@@ -1371,14 +1371,14 @@
         <v>2098215</v>
       </c>
       <c r="E9" s="1" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F9" s="1" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="G9" s="1" t="inlineStr">
         <is>
-          <t>CH SET</t>
+          <t>CH-1 DURUM BILGISI</t>
         </is>
       </c>
     </row>
@@ -1403,11 +1403,11 @@
         <v>4</v>
       </c>
       <c r="F10" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G10" s="1" t="inlineStr">
         <is>
-          <t>CH-1 DURUM BILGISI</t>
+          <t>CH-2 DURUM BILGISI</t>
         </is>
       </c>
     </row>
@@ -1432,11 +1432,11 @@
         <v>4</v>
       </c>
       <c r="F11" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G11" s="1" t="inlineStr">
         <is>
-          <t>CH-2 DURUM BILGISI</t>
+          <t>CH-3 DURUM BILGISI</t>
         </is>
       </c>
     </row>
@@ -1461,11 +1461,11 @@
         <v>4</v>
       </c>
       <c r="F12" s="1" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G12" s="1" t="inlineStr">
         <is>
-          <t>CH-3 DURUM BILGISI</t>
+          <t>CH-4 DURUM BILGISI</t>
         </is>
       </c>
     </row>
@@ -1490,11 +1490,11 @@
         <v>4</v>
       </c>
       <c r="F13" s="1" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G13" s="1" t="inlineStr">
         <is>
-          <t>CH-4 DURUM BILGISI</t>
+          <t>CH-5 DURUM BILGISI</t>
         </is>
       </c>
     </row>
@@ -1519,11 +1519,11 @@
         <v>4</v>
       </c>
       <c r="F14" s="1" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G14" s="1" t="inlineStr">
         <is>
-          <t>CH-5 DURUM BILGISI</t>
+          <t>ABS DURUM BILGISI</t>
         </is>
       </c>
     </row>
@@ -1545,14 +1545,14 @@
         <v>2098215</v>
       </c>
       <c r="E15" s="1" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F15" s="1" t="n">
-        <v>8</v>
+        <v>52</v>
       </c>
       <c r="G15" s="1" t="inlineStr">
         <is>
-          <t>ABS DURUM BILGISI</t>
+          <t>KOJEN-1 DURUM BILGISI</t>
         </is>
       </c>
     </row>
@@ -1577,11 +1577,11 @@
         <v>3</v>
       </c>
       <c r="F16" s="1" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="G16" s="1" t="inlineStr">
         <is>
-          <t>KOJEN-1 DURUM BILGISI</t>
+          <t>KOJEN-2 DURUM BILGISI</t>
         </is>
       </c>
     </row>
@@ -1606,11 +1606,11 @@
         <v>3</v>
       </c>
       <c r="F17" s="1" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="G17" s="1" t="inlineStr">
         <is>
-          <t>KOJEN-2 DURUM BILGISI</t>
+          <t>KOJEN-3 DURUM BILGISI</t>
         </is>
       </c>
     </row>
@@ -1635,11 +1635,11 @@
         <v>3</v>
       </c>
       <c r="F18" s="1" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="G18" s="1" t="inlineStr">
         <is>
-          <t>KOJEN-3 DURUM BILGISI</t>
+          <t>KOJEN-4 DURUM BILGISI</t>
         </is>
       </c>
     </row>
@@ -1661,14 +1661,14 @@
         <v>2098215</v>
       </c>
       <c r="E19" s="1" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F19" s="1" t="n">
-        <v>55</v>
+        <v>28</v>
       </c>
       <c r="G19" s="1" t="inlineStr">
         <is>
-          <t>KOJEN-4 DURUM BILGISI</t>
+          <t>MAS-1 SOGUTMA SICAKLIK</t>
         </is>
       </c>
     </row>
@@ -1693,11 +1693,11 @@
         <v>0</v>
       </c>
       <c r="F20" s="1" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="G20" s="1" t="inlineStr">
         <is>
-          <t>MAS-1 SOGUTMA SICAKLIK</t>
+          <t>MAS-2 SOGUTMA SICAKLIK</t>
         </is>
       </c>
     </row>
@@ -1722,11 +1722,11 @@
         <v>0</v>
       </c>
       <c r="F21" s="1" t="n">
-        <v>29</v>
+        <v>4</v>
       </c>
       <c r="G21" s="1" t="inlineStr">
         <is>
-          <t>MAS-2 SOGUTMA SICAKLIK</t>
+          <t>CH-1 INLET SICAKLIK</t>
         </is>
       </c>
     </row>
@@ -1751,11 +1751,11 @@
         <v>0</v>
       </c>
       <c r="F22" s="1" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G22" s="1" t="inlineStr">
         <is>
-          <t>CH-1 INLET SICAKLIK</t>
+          <t>CH-1 OUTLET CIKIS SICAKLIK</t>
         </is>
       </c>
     </row>
@@ -1780,11 +1780,11 @@
         <v>0</v>
       </c>
       <c r="F23" s="1" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="G23" s="1" t="inlineStr">
         <is>
-          <t>CH-1 OUTLET CIKIS SICAKLIK</t>
+          <t>CH-2 INLET SICAKLIK</t>
         </is>
       </c>
     </row>
@@ -1809,11 +1809,11 @@
         <v>0</v>
       </c>
       <c r="F24" s="1" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G24" s="1" t="inlineStr">
         <is>
-          <t>CH-2 INLET SICAKLIK</t>
+          <t>CH-2 OUTLET SICAKLIK</t>
         </is>
       </c>
     </row>
@@ -1838,11 +1838,11 @@
         <v>0</v>
       </c>
       <c r="F25" s="1" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="G25" s="1" t="inlineStr">
         <is>
-          <t>CH-2 OUTLET SICAKLIK</t>
+          <t>CH-3 INLET SICAKLIK</t>
         </is>
       </c>
     </row>
@@ -1867,11 +1867,11 @@
         <v>0</v>
       </c>
       <c r="F26" s="1" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G26" s="1" t="inlineStr">
         <is>
-          <t>CH-3 INLET SICAKLIK</t>
+          <t>CH-3 OUTLET SICAKLIK</t>
         </is>
       </c>
     </row>
@@ -1896,11 +1896,11 @@
         <v>0</v>
       </c>
       <c r="F27" s="1" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="G27" s="1" t="inlineStr">
         <is>
-          <t>CH-3 OUTLET SICAKLIK</t>
+          <t>CH-4 INLET SICAKLIK</t>
         </is>
       </c>
     </row>
@@ -1925,11 +1925,11 @@
         <v>0</v>
       </c>
       <c r="F28" s="1" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G28" s="1" t="inlineStr">
         <is>
-          <t>CH-4 INLET SICAKLIK</t>
+          <t>CH-4 OUTLET SICAKLIK</t>
         </is>
       </c>
     </row>
@@ -1954,11 +1954,11 @@
         <v>0</v>
       </c>
       <c r="F29" s="1" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="G29" s="1" t="inlineStr">
         <is>
-          <t>CH-4 OUTLET SICAKLIK</t>
+          <t>CH-5 INLET SICAKLIK</t>
         </is>
       </c>
     </row>
@@ -1983,11 +1983,11 @@
         <v>0</v>
       </c>
       <c r="F30" s="1" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G30" s="1" t="inlineStr">
         <is>
-          <t>CH-5 INLET SICAKLIK</t>
+          <t>CH-5 OUTLET CIKIS SICAKLIK</t>
         </is>
       </c>
     </row>
@@ -2012,11 +2012,11 @@
         <v>0</v>
       </c>
       <c r="F31" s="1" t="n">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="G31" s="1" t="inlineStr">
         <is>
-          <t>CH-5 OUTLET CIKIS SICAKLIK</t>
+          <t>ABS INLET SICAKLIK</t>
         </is>
       </c>
     </row>
@@ -2041,69 +2041,69 @@
         <v>0</v>
       </c>
       <c r="F32" s="1" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G32" s="1" t="inlineStr">
         <is>
-          <t>ABS INLET SICAKLIK</t>
+          <t>ABS OUTLET SICAKLIK</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t>192.168.0.2</t>
+          <t>192.168.0.5</t>
         </is>
       </c>
       <c r="B33" s="1" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C33" s="1" t="inlineStr">
         <is>
-          <t>0x0103</t>
+          <t>0x0120</t>
         </is>
       </c>
       <c r="D33" s="1" t="n">
-        <v>2098215</v>
+        <v>2098225</v>
       </c>
       <c r="E33" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F33" s="1" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="G33" s="1" t="inlineStr">
         <is>
-          <t>ABS OUTLET SICAKLIK</t>
+          <t>MAS-2 KAZAN SICAKLIK</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
         <is>
-          <t>192.168.0.5</t>
-        </is>
-      </c>
-      <c r="B34" s="1" t="n">
-        <v>5</v>
-      </c>
-      <c r="C34" s="1" t="inlineStr">
-        <is>
-          <t>0x0120</t>
-        </is>
-      </c>
-      <c r="D34" s="1" t="n">
-        <v>2098225</v>
-      </c>
-      <c r="E34" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="F34" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="G34" s="1" t="inlineStr">
-        <is>
-          <t>MAS-2 KAZAN SICAKLIK</t>
+          <t>192.168.0.2</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>0x011F</t>
+        </is>
+      </c>
+      <c r="D34" s="6" t="n">
+        <v>2098214</v>
+      </c>
+      <c r="E34" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F34" s="7" t="n">
+        <v>378</v>
+      </c>
+      <c r="G34" s="7" t="inlineStr">
+        <is>
+          <t>CH-1 CALISMA YUZDELIK</t>
         </is>
       </c>
     </row>
@@ -2125,14 +2125,14 @@
         <v>2098214</v>
       </c>
       <c r="E35" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F35" s="7" t="n">
-        <v>378</v>
+        <v>27</v>
       </c>
       <c r="G35" s="7" t="inlineStr">
         <is>
-          <t>CH-1 CALISMA YUZDELIK</t>
+          <t>CH-1 IC SET</t>
         </is>
       </c>
     </row>
@@ -2154,14 +2154,14 @@
         <v>2098214</v>
       </c>
       <c r="E36" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F36" s="7" t="n">
-        <v>27</v>
+        <v>398</v>
       </c>
       <c r="G36" s="7" t="inlineStr">
         <is>
-          <t>CH-1 IC SET</t>
+          <t>CH-2 CALISMA YUZDELIK</t>
         </is>
       </c>
     </row>
@@ -2183,14 +2183,14 @@
         <v>2098214</v>
       </c>
       <c r="E37" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F37" s="7" t="n">
-        <v>398</v>
+        <v>29</v>
       </c>
       <c r="G37" s="7" t="inlineStr">
         <is>
-          <t>CH-2 CALISMA YUZDELIK</t>
+          <t>CH-2 IC SET</t>
         </is>
       </c>
     </row>
@@ -2212,14 +2212,14 @@
         <v>2098214</v>
       </c>
       <c r="E38" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F38" s="7" t="n">
-        <v>29</v>
+        <v>418</v>
       </c>
       <c r="G38" s="7" t="inlineStr">
         <is>
-          <t>CH-2 IC SET</t>
+          <t>CH-3 CALISMA YUZDELIK</t>
         </is>
       </c>
     </row>
@@ -2241,14 +2241,14 @@
         <v>2098214</v>
       </c>
       <c r="E39" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F39" s="7" t="n">
-        <v>418</v>
+        <v>31</v>
       </c>
       <c r="G39" s="7" t="inlineStr">
         <is>
-          <t>CH-3 CALISMA YUZDELIK</t>
+          <t>CH-3 IC SET</t>
         </is>
       </c>
     </row>
@@ -2270,14 +2270,14 @@
         <v>2098214</v>
       </c>
       <c r="E40" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F40" s="7" t="n">
-        <v>31</v>
+        <v>344</v>
       </c>
       <c r="G40" s="7" t="inlineStr">
         <is>
-          <t>CH-3 IC SET</t>
+          <t>CH-4 CALISMA YUZDELIK</t>
         </is>
       </c>
     </row>
@@ -2302,11 +2302,11 @@
         <v>0</v>
       </c>
       <c r="F41" s="7" t="n">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="G41" s="7" t="inlineStr">
         <is>
-          <t>CH-4 CALISMA YUZDELIK</t>
+          <t>CH-4 IC SET</t>
         </is>
       </c>
     </row>
@@ -2331,11 +2331,11 @@
         <v>0</v>
       </c>
       <c r="F42" s="7" t="n">
-        <v>346</v>
+        <v>361</v>
       </c>
       <c r="G42" s="7" t="inlineStr">
         <is>
-          <t>CH-4 IC SET</t>
+          <t>CH-5 CALISMA YUZDELIK</t>
         </is>
       </c>
     </row>
@@ -2360,69 +2360,69 @@
         <v>0</v>
       </c>
       <c r="F43" s="7" t="n">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="G43" s="7" t="inlineStr">
         <is>
-          <t>CH-5 CALISMA YUZDELIK</t>
+          <t>CH-5 IC SET</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="4" t="inlineStr">
         <is>
-          <t>192.168.0.2</t>
-        </is>
-      </c>
-      <c r="B44" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="C44" s="5" t="inlineStr">
-        <is>
-          <t>0x011F</t>
-        </is>
-      </c>
-      <c r="D44" s="6" t="n">
-        <v>2098214</v>
-      </c>
-      <c r="E44" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="F44" s="7" t="n">
-        <v>363</v>
-      </c>
-      <c r="G44" s="7" t="inlineStr">
-        <is>
-          <t>CH-5 IC SET</t>
+          <t>192.168.0.4</t>
+        </is>
+      </c>
+      <c r="B44" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="C44" s="1" t="inlineStr">
+        <is>
+          <t>0x0104</t>
+        </is>
+      </c>
+      <c r="D44" s="1" t="n">
+        <v>2099291</v>
+      </c>
+      <c r="E44" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F44" s="1" t="n">
+        <v>25</v>
+      </c>
+      <c r="G44" s="1" t="inlineStr">
+        <is>
+          <t>MAS-1 KAZAN SICAKLIK</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="4" t="inlineStr">
-        <is>
-          <t>192.168.0.4</t>
-        </is>
-      </c>
-      <c r="B45" s="1" t="n">
-        <v>4</v>
-      </c>
-      <c r="C45" s="1" t="inlineStr">
-        <is>
-          <t>0x0104</t>
-        </is>
-      </c>
-      <c r="D45" s="1" t="n">
-        <v>2099291</v>
-      </c>
-      <c r="E45" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="F45" s="1" t="n">
-        <v>25</v>
-      </c>
-      <c r="G45" s="1" t="inlineStr">
-        <is>
-          <t>MAS-1 KAZAN SICAKLIK</t>
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>192.168.0.2</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>2</v>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>0x0103</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>2098215</v>
+      </c>
+      <c r="E45" t="n">
+        <v>0</v>
+      </c>
+      <c r="F45" t="n">
+        <v>34</v>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>KOLLEKTOR SOGUTMA DONUS SICAKLIK</t>
         </is>
       </c>
     </row>
@@ -2437,21 +2437,21 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>0x0103</t>
+          <t>0x011C</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>2098215</v>
+        <v>2098211</v>
       </c>
       <c r="E46" t="n">
         <v>0</v>
       </c>
       <c r="F46" t="n">
-        <v>34</v>
+        <v>14</v>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>KOLLEKTOR SOGUTMA DONUS SICAKLIK</t>
+          <t>KOLLEKTOR ISITMA DONUS SICAKLIK</t>
         </is>
       </c>
     </row>
@@ -2476,11 +2476,11 @@
         <v>0</v>
       </c>
       <c r="F47" t="n">
-        <v>14</v>
+        <v>29</v>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>KOLLEKTOR ISITMA DONUS SICAKLIK</t>
+          <t>KAZAN-1 INLET</t>
         </is>
       </c>
     </row>
@@ -2505,11 +2505,11 @@
         <v>0</v>
       </c>
       <c r="F48" t="n">
-        <v>29</v>
+        <v>16</v>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>KAZAN-1 INLET</t>
+          <t>KAZAN-1 OUTLET</t>
         </is>
       </c>
     </row>
@@ -2534,11 +2534,11 @@
         <v>0</v>
       </c>
       <c r="F49" t="n">
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>KAZAN-1 OUTLET</t>
+          <t>KAZAN-2 INLET</t>
         </is>
       </c>
     </row>
@@ -2563,11 +2563,11 @@
         <v>0</v>
       </c>
       <c r="F50" t="n">
-        <v>30</v>
+        <v>17</v>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>KAZAN-2 INLET</t>
+          <t>KAZAN-2 OUTLET</t>
         </is>
       </c>
     </row>
@@ -2592,11 +2592,11 @@
         <v>0</v>
       </c>
       <c r="F51" t="n">
-        <v>17</v>
+        <v>31</v>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>KAZAN-2 OUTLET</t>
+          <t>KAZAN-3 INLET</t>
         </is>
       </c>
     </row>
@@ -2621,38 +2621,9 @@
         <v>0</v>
       </c>
       <c r="F52" t="n">
-        <v>31</v>
+        <v>18</v>
       </c>
       <c r="G52" t="inlineStr">
-        <is>
-          <t>KAZAN-3 INLET</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>192.168.0.2</t>
-        </is>
-      </c>
-      <c r="B53" t="n">
-        <v>2</v>
-      </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>0x011C</t>
-        </is>
-      </c>
-      <c r="D53" t="n">
-        <v>2098211</v>
-      </c>
-      <c r="E53" t="n">
-        <v>0</v>
-      </c>
-      <c r="F53" t="n">
-        <v>18</v>
-      </c>
-      <c r="G53" t="inlineStr">
         <is>
           <t>KAZAN-3 OUTLET</t>
         </is>

</xml_diff>